<commit_message>
update copy excel sheet
</commit_message>
<xml_diff>
--- a/My_Copy_data_architect_practical_tracker_v6.xlsx
+++ b/My_Copy_data_architect_practical_tracker_v6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dr.Mohammed\OnLine_Courses\DataArchi\data-architecture-course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241D3280-F2B7-48E8-92F8-66B8BBD1474B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DC6102-576E-427E-97DA-1193BB9A4134}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -2211,7 +2211,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2252,6 +2251,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3019,18 +3019,18 @@
       <c r="B2" s="23">
         <v>12</v>
       </c>
-      <c r="C2" s="31">
+      <c r="C2" s="30">
         <f>Dashboard!$B$4+B2*7-3</f>
         <v>46395</v>
       </c>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="28" t="s">
+      <c r="D2" s="28"/>
+      <c r="E2" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="G2" s="40">
+      <c r="G2" s="39">
         <f>Dashboard!$B$4+(7-1)*7</f>
         <v>46356</v>
       </c>
@@ -3042,18 +3042,18 @@
       <c r="B3" s="23">
         <v>17</v>
       </c>
-      <c r="C3" s="31">
+      <c r="C3" s="30">
         <f>Dashboard!$B$4+B3*7-3</f>
         <v>46430</v>
       </c>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="F3" s="28" t="s">
+      <c r="D3" s="28"/>
+      <c r="E3" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="G3" s="40">
+      <c r="G3" s="39">
         <f>Dashboard!$B$4+(13-1)*7</f>
         <v>46398</v>
       </c>
@@ -3065,18 +3065,18 @@
       <c r="B4" s="23">
         <v>21</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="30">
         <f>Dashboard!$B$4+B4*7-3</f>
         <v>46458</v>
       </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="27" t="s">
         <v>300</v>
       </c>
-      <c r="G4" s="40">
+      <c r="G4" s="39">
         <f>Dashboard!$B$4+(18-1)*7</f>
         <v>46433</v>
       </c>
@@ -3088,18 +3088,18 @@
       <c r="B5" s="23">
         <v>6</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="30">
         <f>Dashboard!$B$4+B5*7-3</f>
         <v>46353</v>
       </c>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="F5" s="28" t="s">
+      <c r="D5" s="28"/>
+      <c r="E5" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="G5" s="40">
+      <c r="G5" s="39">
         <f>Dashboard!$B$4+(3-1)*7</f>
         <v>46328</v>
       </c>
@@ -3165,22 +3165,22 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="28" t="s">
         <v>640</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="28" t="s">
         <v>641</v>
       </c>
-      <c r="C2" s="38">
+      <c r="C2" s="37">
         <v>46370</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="28" t="s">
         <v>642</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="28" t="s">
         <v>643</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="28" t="s">
         <v>644</v>
       </c>
       <c r="H2" s="6" t="s">
@@ -3188,254 +3188,254 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
       <c r="H3" s="6" t="s">
         <v>641</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="29"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="H4" s="6" t="s">
         <v>646</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="29"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
       <c r="H5" s="6" t="s">
         <v>647</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
       <c r="H6" s="6" t="s">
         <v>648</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
       <c r="H7" s="6" t="s">
         <v>649</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
       <c r="H9" s="2" t="s">
         <v>650</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="29"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
+      <c r="A28" s="28"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
+      <c r="A29" s="28"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="29"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3585,7 +3585,7 @@
       <c r="A17" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="27" t="str">
+      <c r="B17" s="41" t="str">
         <f ca="1">HYPERLINK(INDEX('Weekly Plan'!$F$2:$F$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)),"Open the main link")</f>
         <v>Open the main link</v>
       </c>
@@ -3594,7 +3594,7 @@
       <c r="A18" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="28" t="str">
+      <c r="B18" s="27" t="str">
         <f ca="1">IF(INDEX('Weekly Plan'!$Q$2:$Q$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0))="","",IF(INDEX('Weekly Plan'!$R$2:$R$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0))="",INDEX('Weekly Plan'!$Q$2:$Q$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)),HYPERLINK(INDEX('Weekly Plan'!$R$2:$R$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)),INDEX('Weekly Plan'!$Q$2:$Q$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)))))</f>
         <v>Microsoft Learn: Understand star schema</v>
       </c>
@@ -3603,7 +3603,7 @@
       <c r="A19" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="28" t="str">
+      <c r="B19" s="27" t="str">
         <f ca="1">IF(INDEX('Weekly Plan'!$S$2:$S$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0))="","",IF(INDEX('Weekly Plan'!$T$2:$T$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0))="",INDEX('Weekly Plan'!$S$2:$S$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)),HYPERLINK(INDEX('Weekly Plan'!$T$2:$T$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)),INDEX('Weekly Plan'!$S$2:$S$24,MATCH($B$5,'Weekly Plan'!$A$2:$A$24,0)))))</f>
         <v>Book: The Data Warehouse Toolkit (Kimball and Ross), ch. 1-3 (borrow)</v>
       </c>
@@ -3632,7 +3632,7 @@
         <f ca="1">"Learn: "&amp;B10</f>
         <v>Learn: Coginiti: Dimensional Modeling and the Star Schema (guide)</v>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="28">
         <v>1.5</v>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
         <f ca="1">"Learn: "&amp;IF(B18="",B10,B18)</f>
         <v>Learn: Microsoft Learn: Understand star schema</v>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="28">
         <v>1.5</v>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       <c r="B25" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="28">
         <v>2</v>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       <c r="B26" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="29">
+      <c r="C26" s="28">
         <v>1.5</v>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
       <c r="B27" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="28">
         <v>3</v>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
       <c r="B28" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="29">
+      <c r="C28" s="28">
         <v>0.5</v>
       </c>
     </row>
@@ -3777,13 +3777,13 @@
       <c r="B2" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="29"/>
+      <c r="D2" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="28"/>
     </row>
     <row r="3" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="23">
@@ -3793,10 +3793,10 @@
         <v>85</v>
       </c>
       <c r="C3" s="23"/>
-      <c r="D3" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="29"/>
+      <c r="D3" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="28"/>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="23">
@@ -3805,13 +3805,13 @@
       <c r="B4" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="40" t="s">
         <v>653</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="28" t="s">
         <v>651</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="28"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="23">
@@ -3821,10 +3821,10 @@
         <v>87</v>
       </c>
       <c r="C5" s="23"/>
-      <c r="D5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="29"/>
+      <c r="D5" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="23">
@@ -3833,13 +3833,13 @@
       <c r="B6" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="28" t="s">
         <v>651</v>
       </c>
-      <c r="E6" s="29"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="23">
@@ -3848,13 +3848,13 @@
       <c r="B7" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="28" t="s">
         <v>651</v>
       </c>
-      <c r="E7" s="29"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="23">
@@ -3863,13 +3863,13 @@
       <c r="B8" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="29"/>
+      <c r="D8" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="23">
@@ -3878,13 +3878,13 @@
       <c r="B9" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="D9" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" s="29"/>
+      <c r="D9" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="23">
@@ -3896,10 +3896,10 @@
       <c r="C10" s="23" t="s">
         <v>652</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="28" t="s">
         <v>651</v>
       </c>
-      <c r="E10" s="29"/>
+      <c r="E10" s="28"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="23">
@@ -3909,10 +3909,10 @@
         <v>97</v>
       </c>
       <c r="C11" s="23"/>
-      <c r="D11" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" s="29"/>
+      <c r="D11" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="28"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D11">
@@ -4031,14 +4031,14 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="30">
+      <c r="A2" s="29">
         <v>1</v>
       </c>
-      <c r="B2" s="31">
+      <c r="B2" s="30">
         <f>Dashboard!$B$4+(A2-1)*7</f>
         <v>46314</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="29" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
@@ -4047,7 +4047,7 @@
       <c r="E2" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="27" t="s">
         <v>112</v>
       </c>
       <c r="G2" s="23" t="s">
@@ -4063,21 +4063,21 @@
       <c r="K2" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="L2" s="32">
+      <c r="L2" s="31">
         <v>4</v>
       </c>
-      <c r="M2" s="32">
+      <c r="M2" s="31">
         <v>6</v>
       </c>
-      <c r="N2" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
+      <c r="N2" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
       <c r="Q2" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="R2" s="27" t="s">
         <v>118</v>
       </c>
       <c r="S2" s="23" t="s">
@@ -4086,14 +4086,14 @@
       <c r="T2" s="23"/>
     </row>
     <row r="3" spans="1:20" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="30">
+      <c r="A3" s="29">
         <v>2</v>
       </c>
-      <c r="B3" s="31">
+      <c r="B3" s="30">
         <f>Dashboard!$B$4+(A3-1)*7</f>
         <v>46321</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="29" t="s">
         <v>23</v>
       </c>
       <c r="D3" s="23" t="s">
@@ -4102,7 +4102,7 @@
       <c r="E3" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="27" t="s">
         <v>122</v>
       </c>
       <c r="G3" s="23" t="s">
@@ -4118,39 +4118,39 @@
       <c r="K3" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="L3" s="32">
+      <c r="L3" s="31">
         <v>4</v>
       </c>
-      <c r="M3" s="32">
+      <c r="M3" s="31">
         <v>6</v>
       </c>
-      <c r="N3" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
+      <c r="N3" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
       <c r="Q3" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="R3" s="28" t="s">
+      <c r="R3" s="27" t="s">
         <v>128</v>
       </c>
       <c r="S3" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="T3" s="28" t="s">
+      <c r="T3" s="27" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="30">
+      <c r="A4" s="29">
         <v>3</v>
       </c>
-      <c r="B4" s="31">
+      <c r="B4" s="30">
         <f>Dashboard!$B$4+(A4-1)*7</f>
         <v>46328</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="29" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
@@ -4159,7 +4159,7 @@
       <c r="E4" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="27" t="s">
         <v>133</v>
       </c>
       <c r="G4" s="23" t="s">
@@ -4177,39 +4177,39 @@
       <c r="K4" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="L4" s="32">
+      <c r="L4" s="31">
         <v>4</v>
       </c>
-      <c r="M4" s="32">
+      <c r="M4" s="31">
         <v>6</v>
       </c>
-      <c r="N4" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
+      <c r="N4" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
       <c r="Q4" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="27" t="s">
         <v>140</v>
       </c>
       <c r="S4" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="T4" s="28" t="s">
+      <c r="T4" s="27" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="33">
+      <c r="A5" s="32">
         <v>4</v>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="30">
         <f>Dashboard!$B$4+(A5-1)*7</f>
         <v>46335</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="32" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="23" t="s">
@@ -4218,7 +4218,7 @@
       <c r="E5" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="F5" s="27" t="s">
         <v>83</v>
       </c>
       <c r="G5" s="23" t="s">
@@ -4234,39 +4234,39 @@
       <c r="K5" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="L5" s="32">
+      <c r="L5" s="31">
         <v>5</v>
       </c>
-      <c r="M5" s="32">
+      <c r="M5" s="31">
         <v>5</v>
       </c>
-      <c r="N5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O5" s="29"/>
-      <c r="P5" s="29"/>
+      <c r="N5" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
       <c r="Q5" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="R5" s="28" t="s">
+      <c r="R5" s="27" t="s">
         <v>150</v>
       </c>
       <c r="S5" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="T5" s="28" t="s">
+      <c r="T5" s="27" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="33">
+      <c r="A6" s="32">
         <v>5</v>
       </c>
-      <c r="B6" s="31">
+      <c r="B6" s="30">
         <f>Dashboard!$B$4+(A6-1)*7</f>
         <v>46342</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="32" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="23" t="s">
@@ -4275,7 +4275,7 @@
       <c r="E6" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="F6" s="28" t="s">
+      <c r="F6" s="27" t="s">
         <v>155</v>
       </c>
       <c r="G6" s="23" t="s">
@@ -4291,39 +4291,39 @@
       <c r="K6" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="L6" s="32">
+      <c r="L6" s="31">
         <v>5</v>
       </c>
-      <c r="M6" s="32">
+      <c r="M6" s="31">
         <v>5</v>
       </c>
-      <c r="N6" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O6" s="29"/>
-      <c r="P6" s="29"/>
+      <c r="N6" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
       <c r="Q6" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="R6" s="28" t="s">
+      <c r="R6" s="27" t="s">
         <v>150</v>
       </c>
       <c r="S6" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="T6" s="28" t="s">
+      <c r="T6" s="27" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="66" x14ac:dyDescent="0.3">
-      <c r="A7" s="33">
+      <c r="A7" s="32">
         <v>6</v>
       </c>
-      <c r="B7" s="31">
+      <c r="B7" s="30">
         <f>Dashboard!$B$4+(A7-1)*7</f>
         <v>46349</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="32" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="23" t="s">
@@ -4332,7 +4332,7 @@
       <c r="E7" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="F7" s="28"/>
+      <c r="F7" s="27"/>
       <c r="G7" s="23" t="s">
         <v>164</v>
       </c>
@@ -4348,39 +4348,39 @@
       <c r="K7" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="L7" s="32">
+      <c r="L7" s="31">
         <v>6</v>
       </c>
-      <c r="M7" s="32">
+      <c r="M7" s="31">
         <v>4</v>
       </c>
-      <c r="N7" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O7" s="29"/>
-      <c r="P7" s="29"/>
+      <c r="N7" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
       <c r="Q7" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="R7" s="28" t="s">
+      <c r="R7" s="27" t="s">
         <v>83</v>
       </c>
       <c r="S7" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="T7" s="28" t="s">
+      <c r="T7" s="27" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="34">
+      <c r="A8" s="33">
         <v>7</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="30">
         <f>Dashboard!$B$4+(A8-1)*7</f>
         <v>46356</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D8" s="23" t="s">
@@ -4389,7 +4389,7 @@
       <c r="E8" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="27" t="s">
         <v>173</v>
       </c>
       <c r="G8" s="23" t="s">
@@ -4407,39 +4407,39 @@
       <c r="K8" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="L8" s="32">
+      <c r="L8" s="31">
         <v>4</v>
       </c>
-      <c r="M8" s="32">
+      <c r="M8" s="31">
         <v>6</v>
       </c>
-      <c r="N8" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O8" s="29"/>
-      <c r="P8" s="29"/>
+      <c r="N8" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
       <c r="Q8" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="R8" s="28" t="s">
+      <c r="R8" s="27" t="s">
         <v>150</v>
       </c>
       <c r="S8" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="T8" s="28" t="s">
+      <c r="T8" s="27" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="34">
+      <c r="A9" s="33">
         <v>8</v>
       </c>
-      <c r="B9" s="31">
+      <c r="B9" s="30">
         <f>Dashboard!$B$4+(A9-1)*7</f>
         <v>46363</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="23" t="s">
@@ -4448,7 +4448,7 @@
       <c r="E9" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="27" t="s">
         <v>155</v>
       </c>
       <c r="G9" s="23" t="s">
@@ -4464,39 +4464,39 @@
       <c r="K9" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="L9" s="32">
+      <c r="L9" s="31">
         <v>4</v>
       </c>
-      <c r="M9" s="32">
+      <c r="M9" s="31">
         <v>6</v>
       </c>
-      <c r="N9" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O9" s="29"/>
-      <c r="P9" s="29"/>
+      <c r="N9" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
       <c r="Q9" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="R9" s="28" t="s">
+      <c r="R9" s="27" t="s">
         <v>150</v>
       </c>
       <c r="S9" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="T9" s="28" t="s">
+      <c r="T9" s="27" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="34">
+      <c r="A10" s="33">
         <v>9</v>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="30">
         <f>Dashboard!$B$4+(A10-1)*7</f>
         <v>46370</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="23" t="s">
@@ -4505,7 +4505,7 @@
       <c r="E10" s="23" t="s">
         <v>191</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="27" t="s">
         <v>192</v>
       </c>
       <c r="G10" s="23" t="s">
@@ -4521,39 +4521,39 @@
       <c r="K10" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="31">
         <v>4</v>
       </c>
-      <c r="M10" s="32">
+      <c r="M10" s="31">
         <v>6</v>
       </c>
-      <c r="N10" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O10" s="29"/>
-      <c r="P10" s="29"/>
+      <c r="N10" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
       <c r="Q10" s="23" t="s">
         <v>197</v>
       </c>
-      <c r="R10" s="28" t="s">
+      <c r="R10" s="27" t="s">
         <v>152</v>
       </c>
       <c r="S10" s="23" t="s">
         <v>198</v>
       </c>
-      <c r="T10" s="28" t="s">
+      <c r="T10" s="27" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="34">
+      <c r="A11" s="33">
         <v>10</v>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="30">
         <f>Dashboard!$B$4+(A11-1)*7</f>
         <v>46377</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="23" t="s">
@@ -4562,7 +4562,7 @@
       <c r="E11" s="23" t="s">
         <v>200</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="27" t="s">
         <v>150</v>
       </c>
       <c r="G11" s="23" t="s">
@@ -4578,39 +4578,39 @@
       <c r="K11" s="23" t="s">
         <v>204</v>
       </c>
-      <c r="L11" s="32">
+      <c r="L11" s="31">
         <v>4</v>
       </c>
-      <c r="M11" s="32">
+      <c r="M11" s="31">
         <v>6</v>
       </c>
-      <c r="N11" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O11" s="29"/>
-      <c r="P11" s="29"/>
+      <c r="N11" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O11" s="28"/>
+      <c r="P11" s="28"/>
       <c r="Q11" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="R11" s="28" t="s">
+      <c r="R11" s="27" t="s">
         <v>206</v>
       </c>
       <c r="S11" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="T11" s="28" t="s">
+      <c r="T11" s="27" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="34">
+      <c r="A12" s="33">
         <v>11</v>
       </c>
-      <c r="B12" s="31">
+      <c r="B12" s="30">
         <f>Dashboard!$B$4+(A12-1)*7</f>
         <v>46384</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D12" s="23" t="s">
@@ -4619,7 +4619,7 @@
       <c r="E12" s="23" t="s">
         <v>209</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="27" t="s">
         <v>210</v>
       </c>
       <c r="G12" s="23" t="s">
@@ -4635,39 +4635,39 @@
       <c r="K12" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="L12" s="32">
+      <c r="L12" s="31">
         <v>4</v>
       </c>
-      <c r="M12" s="32">
+      <c r="M12" s="31">
         <v>6</v>
       </c>
-      <c r="N12" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O12" s="29"/>
-      <c r="P12" s="29"/>
+      <c r="N12" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O12" s="28"/>
+      <c r="P12" s="28"/>
       <c r="Q12" s="23" t="s">
         <v>215</v>
       </c>
-      <c r="R12" s="28" t="s">
+      <c r="R12" s="27" t="s">
         <v>152</v>
       </c>
       <c r="S12" s="23" t="s">
         <v>216</v>
       </c>
-      <c r="T12" s="28" t="s">
+      <c r="T12" s="27" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="34">
+      <c r="A13" s="33">
         <v>12</v>
       </c>
-      <c r="B13" s="31">
+      <c r="B13" s="30">
         <f>Dashboard!$B$4+(A13-1)*7</f>
         <v>46391</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="33" t="s">
         <v>25</v>
       </c>
       <c r="D13" s="23" t="s">
@@ -4676,7 +4676,7 @@
       <c r="E13" s="23" t="s">
         <v>219</v>
       </c>
-      <c r="F13" s="28"/>
+      <c r="F13" s="27"/>
       <c r="G13" s="23" t="s">
         <v>220</v>
       </c>
@@ -4692,39 +4692,39 @@
       <c r="K13" s="23" t="s">
         <v>224</v>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="31">
         <v>6</v>
       </c>
-      <c r="M13" s="32">
+      <c r="M13" s="31">
         <v>4</v>
       </c>
-      <c r="N13" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O13" s="29"/>
-      <c r="P13" s="29"/>
+      <c r="N13" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O13" s="28"/>
+      <c r="P13" s="28"/>
       <c r="Q13" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="R13" s="28" t="s">
+      <c r="R13" s="27" t="s">
         <v>173</v>
       </c>
       <c r="S13" s="23" t="s">
         <v>226</v>
       </c>
-      <c r="T13" s="28" t="s">
+      <c r="T13" s="27" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="35">
+      <c r="A14" s="34">
         <v>13</v>
       </c>
-      <c r="B14" s="31">
+      <c r="B14" s="30">
         <f>Dashboard!$B$4+(A14-1)*7</f>
         <v>46398</v>
       </c>
-      <c r="C14" s="35" t="s">
+      <c r="C14" s="34" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="23" t="s">
@@ -4733,7 +4733,7 @@
       <c r="E14" s="23" t="s">
         <v>229</v>
       </c>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="27" t="s">
         <v>230</v>
       </c>
       <c r="G14" s="23" t="s">
@@ -4751,39 +4751,39 @@
       <c r="K14" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="L14" s="32">
+      <c r="L14" s="31">
         <v>4</v>
       </c>
-      <c r="M14" s="32">
+      <c r="M14" s="31">
         <v>6</v>
       </c>
-      <c r="N14" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O14" s="29"/>
-      <c r="P14" s="29"/>
+      <c r="N14" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O14" s="28"/>
+      <c r="P14" s="28"/>
       <c r="Q14" s="23" t="s">
         <v>236</v>
       </c>
-      <c r="R14" s="28" t="s">
+      <c r="R14" s="27" t="s">
         <v>237</v>
       </c>
       <c r="S14" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="T14" s="28" t="s">
+      <c r="T14" s="27" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="35">
+      <c r="A15" s="34">
         <v>14</v>
       </c>
-      <c r="B15" s="31">
+      <c r="B15" s="30">
         <f>Dashboard!$B$4+(A15-1)*7</f>
         <v>46405</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="34" t="s">
         <v>26</v>
       </c>
       <c r="D15" s="23" t="s">
@@ -4792,7 +4792,7 @@
       <c r="E15" s="23" t="s">
         <v>241</v>
       </c>
-      <c r="F15" s="28" t="s">
+      <c r="F15" s="27" t="s">
         <v>230</v>
       </c>
       <c r="G15" s="23" t="s">
@@ -4808,39 +4808,39 @@
       <c r="K15" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="L15" s="32">
+      <c r="L15" s="31">
         <v>4</v>
       </c>
-      <c r="M15" s="32">
+      <c r="M15" s="31">
         <v>6</v>
       </c>
-      <c r="N15" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O15" s="29"/>
-      <c r="P15" s="29"/>
+      <c r="N15" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O15" s="28"/>
+      <c r="P15" s="28"/>
       <c r="Q15" s="23" t="s">
         <v>246</v>
       </c>
-      <c r="R15" s="28" t="s">
+      <c r="R15" s="27" t="s">
         <v>247</v>
       </c>
       <c r="S15" s="23" t="s">
         <v>248</v>
       </c>
-      <c r="T15" s="28" t="s">
+      <c r="T15" s="27" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="35">
+      <c r="A16" s="34">
         <v>15</v>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="30">
         <f>Dashboard!$B$4+(A16-1)*7</f>
         <v>46412</v>
       </c>
-      <c r="C16" s="35" t="s">
+      <c r="C16" s="34" t="s">
         <v>26</v>
       </c>
       <c r="D16" s="23" t="s">
@@ -4849,7 +4849,7 @@
       <c r="E16" s="23" t="s">
         <v>251</v>
       </c>
-      <c r="F16" s="28" t="s">
+      <c r="F16" s="27" t="s">
         <v>230</v>
       </c>
       <c r="G16" s="23" t="s">
@@ -4865,21 +4865,21 @@
       <c r="K16" s="23" t="s">
         <v>255</v>
       </c>
-      <c r="L16" s="32">
+      <c r="L16" s="31">
         <v>4</v>
       </c>
-      <c r="M16" s="32">
+      <c r="M16" s="31">
         <v>6</v>
       </c>
-      <c r="N16" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
+      <c r="N16" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O16" s="28"/>
+      <c r="P16" s="28"/>
       <c r="Q16" s="23" t="s">
         <v>256</v>
       </c>
-      <c r="R16" s="28" t="s">
+      <c r="R16" s="27" t="s">
         <v>257</v>
       </c>
       <c r="S16" s="23" t="s">
@@ -4888,14 +4888,14 @@
       <c r="T16" s="23"/>
     </row>
     <row r="17" spans="1:20" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="35">
+      <c r="A17" s="34">
         <v>16</v>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="30">
         <f>Dashboard!$B$4+(A17-1)*7</f>
         <v>46419</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="34" t="s">
         <v>26</v>
       </c>
       <c r="D17" s="23" t="s">
@@ -4904,7 +4904,7 @@
       <c r="E17" s="23" t="s">
         <v>260</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="27" t="s">
         <v>230</v>
       </c>
       <c r="G17" s="23" t="s">
@@ -4920,39 +4920,39 @@
       <c r="K17" s="23" t="s">
         <v>263</v>
       </c>
-      <c r="L17" s="32">
+      <c r="L17" s="31">
         <v>4</v>
       </c>
-      <c r="M17" s="32">
+      <c r="M17" s="31">
         <v>6</v>
       </c>
-      <c r="N17" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O17" s="29"/>
-      <c r="P17" s="29"/>
+      <c r="N17" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O17" s="28"/>
+      <c r="P17" s="28"/>
       <c r="Q17" s="23" t="s">
         <v>264</v>
       </c>
-      <c r="R17" s="28" t="s">
+      <c r="R17" s="27" t="s">
         <v>265</v>
       </c>
       <c r="S17" s="23" t="s">
         <v>266</v>
       </c>
-      <c r="T17" s="28" t="s">
+      <c r="T17" s="27" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="35">
+      <c r="A18" s="34">
         <v>17</v>
       </c>
-      <c r="B18" s="31">
+      <c r="B18" s="30">
         <f>Dashboard!$B$4+(A18-1)*7</f>
         <v>46426</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="34" t="s">
         <v>26</v>
       </c>
       <c r="D18" s="23" t="s">
@@ -4961,7 +4961,7 @@
       <c r="E18" s="23" t="s">
         <v>269</v>
       </c>
-      <c r="F18" s="28"/>
+      <c r="F18" s="27"/>
       <c r="G18" s="23" t="s">
         <v>270</v>
       </c>
@@ -4977,39 +4977,39 @@
       <c r="K18" s="23" t="s">
         <v>274</v>
       </c>
-      <c r="L18" s="32">
+      <c r="L18" s="31">
         <v>6</v>
       </c>
-      <c r="M18" s="32">
+      <c r="M18" s="31">
         <v>4</v>
       </c>
-      <c r="N18" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O18" s="29"/>
-      <c r="P18" s="29"/>
+      <c r="N18" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O18" s="28"/>
+      <c r="P18" s="28"/>
       <c r="Q18" s="23" t="s">
         <v>275</v>
       </c>
-      <c r="R18" s="28" t="s">
+      <c r="R18" s="27" t="s">
         <v>239</v>
       </c>
       <c r="S18" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="T18" s="28" t="s">
+      <c r="T18" s="27" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="36">
+      <c r="A19" s="35">
         <v>18</v>
       </c>
-      <c r="B19" s="31">
+      <c r="B19" s="30">
         <f>Dashboard!$B$4+(A19-1)*7</f>
         <v>46433</v>
       </c>
-      <c r="C19" s="36" t="s">
+      <c r="C19" s="35" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="23" t="s">
@@ -5018,7 +5018,7 @@
       <c r="E19" s="23" t="s">
         <v>279</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="27" t="s">
         <v>280</v>
       </c>
       <c r="G19" s="23" t="s">
@@ -5036,39 +5036,39 @@
       <c r="K19" s="23" t="s">
         <v>285</v>
       </c>
-      <c r="L19" s="32">
+      <c r="L19" s="31">
         <v>4</v>
       </c>
-      <c r="M19" s="32">
+      <c r="M19" s="31">
         <v>6</v>
       </c>
-      <c r="N19" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O19" s="29"/>
-      <c r="P19" s="29"/>
+      <c r="N19" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O19" s="28"/>
+      <c r="P19" s="28"/>
       <c r="Q19" s="23" t="s">
         <v>286</v>
       </c>
-      <c r="R19" s="28" t="s">
+      <c r="R19" s="27" t="s">
         <v>287</v>
       </c>
       <c r="S19" s="23" t="s">
         <v>288</v>
       </c>
-      <c r="T19" s="28" t="s">
+      <c r="T19" s="27" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="20" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="36">
+      <c r="A20" s="35">
         <v>19</v>
       </c>
-      <c r="B20" s="31">
+      <c r="B20" s="30">
         <f>Dashboard!$B$4+(A20-1)*7</f>
         <v>46440</v>
       </c>
-      <c r="C20" s="36" t="s">
+      <c r="C20" s="35" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="23" t="s">
@@ -5077,7 +5077,7 @@
       <c r="E20" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="27" t="s">
         <v>292</v>
       </c>
       <c r="G20" s="23" t="s">
@@ -5093,39 +5093,39 @@
       <c r="K20" s="23" t="s">
         <v>296</v>
       </c>
-      <c r="L20" s="32">
+      <c r="L20" s="31">
         <v>4</v>
       </c>
-      <c r="M20" s="32">
+      <c r="M20" s="31">
         <v>6</v>
       </c>
-      <c r="N20" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O20" s="29"/>
-      <c r="P20" s="29"/>
+      <c r="N20" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
       <c r="Q20" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="R20" s="28" t="s">
+      <c r="R20" s="27" t="s">
         <v>298</v>
       </c>
       <c r="S20" s="23" t="s">
         <v>299</v>
       </c>
-      <c r="T20" s="28" t="s">
+      <c r="T20" s="27" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="21" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="36">
+      <c r="A21" s="35">
         <v>20</v>
       </c>
-      <c r="B21" s="31">
+      <c r="B21" s="30">
         <f>Dashboard!$B$4+(A21-1)*7</f>
         <v>46447</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="35" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="23" t="s">
@@ -5134,7 +5134,7 @@
       <c r="E21" s="23" t="s">
         <v>302</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="27" t="s">
         <v>303</v>
       </c>
       <c r="G21" s="23" t="s">
@@ -5150,39 +5150,39 @@
       <c r="K21" s="23" t="s">
         <v>307</v>
       </c>
-      <c r="L21" s="32">
+      <c r="L21" s="31">
         <v>4</v>
       </c>
-      <c r="M21" s="32">
+      <c r="M21" s="31">
         <v>6</v>
       </c>
-      <c r="N21" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O21" s="29"/>
-      <c r="P21" s="29"/>
+      <c r="N21" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O21" s="28"/>
+      <c r="P21" s="28"/>
       <c r="Q21" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="R21" s="28" t="s">
+      <c r="R21" s="27" t="s">
         <v>309</v>
       </c>
       <c r="S21" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="T21" s="28" t="s">
+      <c r="T21" s="27" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="22" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="36">
+      <c r="A22" s="35">
         <v>21</v>
       </c>
-      <c r="B22" s="31">
+      <c r="B22" s="30">
         <f>Dashboard!$B$4+(A22-1)*7</f>
         <v>46454</v>
       </c>
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="35" t="s">
         <v>27</v>
       </c>
       <c r="D22" s="23" t="s">
@@ -5191,7 +5191,7 @@
       <c r="E22" s="23" t="s">
         <v>313</v>
       </c>
-      <c r="F22" s="28" t="s">
+      <c r="F22" s="27" t="s">
         <v>314</v>
       </c>
       <c r="G22" s="23" t="s">
@@ -5209,17 +5209,17 @@
       <c r="K22" s="23" t="s">
         <v>319</v>
       </c>
-      <c r="L22" s="32">
+      <c r="L22" s="31">
         <v>6</v>
       </c>
-      <c r="M22" s="32">
+      <c r="M22" s="31">
         <v>4</v>
       </c>
-      <c r="N22" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O22" s="29"/>
-      <c r="P22" s="29"/>
+      <c r="N22" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O22" s="28"/>
+      <c r="P22" s="28"/>
       <c r="Q22" s="23" t="s">
         <v>320</v>
       </c>
@@ -5227,19 +5227,19 @@
       <c r="S22" s="23" t="s">
         <v>299</v>
       </c>
-      <c r="T22" s="28" t="s">
+      <c r="T22" s="27" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="37">
+      <c r="A23" s="36">
         <v>22</v>
       </c>
-      <c r="B23" s="31">
+      <c r="B23" s="30">
         <f>Dashboard!$B$4+(A23-1)*7</f>
         <v>46461</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="36" t="s">
         <v>28</v>
       </c>
       <c r="D23" s="23" t="s">
@@ -5248,7 +5248,7 @@
       <c r="E23" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="27" t="s">
         <v>323</v>
       </c>
       <c r="G23" s="23" t="s">
@@ -5264,35 +5264,35 @@
       <c r="K23" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="L23" s="32">
+      <c r="L23" s="31">
         <v>0</v>
       </c>
-      <c r="M23" s="32">
+      <c r="M23" s="31">
         <v>10</v>
       </c>
-      <c r="N23" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O23" s="29"/>
-      <c r="P23" s="29"/>
+      <c r="N23" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
       <c r="Q23" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="R23" s="28" t="s">
+      <c r="R23" s="27" t="s">
         <v>142</v>
       </c>
       <c r="S23" s="23"/>
       <c r="T23" s="23"/>
     </row>
     <row r="24" spans="1:20" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="37">
+      <c r="A24" s="36">
         <v>23</v>
       </c>
-      <c r="B24" s="31">
+      <c r="B24" s="30">
         <f>Dashboard!$B$4+(A24-1)*7</f>
         <v>46468</v>
       </c>
-      <c r="C24" s="37" t="s">
+      <c r="C24" s="36" t="s">
         <v>28</v>
       </c>
       <c r="D24" s="23" t="s">
@@ -5301,7 +5301,7 @@
       <c r="E24" s="23" t="s">
         <v>329</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="27" t="s">
         <v>142</v>
       </c>
       <c r="G24" s="23" t="s">
@@ -5317,17 +5317,17 @@
       <c r="K24" s="23" t="s">
         <v>333</v>
       </c>
-      <c r="L24" s="32">
+      <c r="L24" s="31">
         <v>0</v>
       </c>
-      <c r="M24" s="32">
+      <c r="M24" s="31">
         <v>10</v>
       </c>
-      <c r="N24" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="O24" s="29"/>
-      <c r="P24" s="29"/>
+      <c r="N24" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="O24" s="28"/>
+      <c r="P24" s="28"/>
       <c r="Q24" s="23"/>
       <c r="R24" s="23"/>
       <c r="S24" s="23"/>
@@ -5501,10 +5501,10 @@
       <c r="G2" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="40" t="s">
         <v>112</v>
       </c>
-      <c r="I2" s="29" t="s">
+      <c r="I2" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J2" s="23" t="s">
@@ -5531,10 +5531,10 @@
       <c r="G3" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="I3" s="29" t="s">
+      <c r="I3" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J3" s="23" t="s">
@@ -5562,7 +5562,7 @@
         <v>354</v>
       </c>
       <c r="H4" s="23"/>
-      <c r="I4" s="29" t="s">
+      <c r="I4" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J4" s="23" t="s">
@@ -5589,10 +5589,10 @@
       <c r="G5" s="23" t="s">
         <v>359</v>
       </c>
-      <c r="H5" s="28" t="s">
+      <c r="H5" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="I5" s="29" t="s">
+      <c r="I5" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J5" s="23" t="s">
@@ -5621,10 +5621,10 @@
       <c r="G6" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H6" s="28" t="s">
+      <c r="H6" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="I6" s="29" t="s">
+      <c r="I6" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J6" s="23" t="s">
@@ -5651,10 +5651,10 @@
       <c r="G7" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H7" s="28" t="s">
+      <c r="H7" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="I7" s="29" t="s">
+      <c r="I7" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J7" s="23" t="s">
@@ -5681,10 +5681,10 @@
       <c r="G8" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H8" s="28" t="s">
+      <c r="H8" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="I8" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J8" s="23" t="s">
@@ -5711,10 +5711,10 @@
       <c r="G9" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="I9" s="29" t="s">
+      <c r="I9" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J9" s="23" t="s">
@@ -5741,10 +5741,10 @@
       <c r="G10" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H10" s="28" t="s">
+      <c r="H10" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="I10" s="29" t="s">
+      <c r="I10" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J10" s="23" t="s">
@@ -5771,10 +5771,10 @@
       <c r="G11" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H11" s="28" t="s">
+      <c r="H11" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="I11" s="29" t="s">
+      <c r="I11" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J11" s="23" t="s">
@@ -5801,10 +5801,10 @@
       <c r="G12" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H12" s="28" t="s">
+      <c r="H12" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="I12" s="29" t="s">
+      <c r="I12" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J12" s="23" t="s">
@@ -5833,10 +5833,10 @@
       <c r="G13" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H13" s="28" t="s">
+      <c r="H13" s="27" t="s">
         <v>390</v>
       </c>
-      <c r="I13" s="29" t="s">
+      <c r="I13" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J13" s="23" t="s">
@@ -5865,10 +5865,10 @@
       <c r="G14" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H14" s="28" t="s">
+      <c r="H14" s="27" t="s">
         <v>394</v>
       </c>
-      <c r="I14" s="29" t="s">
+      <c r="I14" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J14" s="23" t="s">
@@ -5897,10 +5897,10 @@
       <c r="G15" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H15" s="28" t="s">
+      <c r="H15" s="27" t="s">
         <v>398</v>
       </c>
-      <c r="I15" s="29" t="s">
+      <c r="I15" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J15" s="23" t="s">
@@ -5927,10 +5927,10 @@
       <c r="G16" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H16" s="28" t="s">
+      <c r="H16" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="I16" s="29" t="s">
+      <c r="I16" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J16" s="23" t="s">
@@ -5957,10 +5957,10 @@
       <c r="G17" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="H17" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="I17" s="29" t="s">
+      <c r="I17" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J17" s="23" t="s">
@@ -5987,10 +5987,10 @@
       <c r="G18" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="I18" s="29" t="s">
+      <c r="I18" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J18" s="23"/>
@@ -6015,10 +6015,10 @@
       <c r="G19" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="I19" s="29" t="s">
+      <c r="I19" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J19" s="23" t="s">
@@ -6047,10 +6047,10 @@
       <c r="G20" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H20" s="28" t="s">
+      <c r="H20" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="I20" s="29" t="s">
+      <c r="I20" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J20" s="23" t="s">
@@ -6077,10 +6077,10 @@
       <c r="G21" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H21" s="28" t="s">
+      <c r="H21" s="27" t="s">
         <v>237</v>
       </c>
-      <c r="I21" s="29" t="s">
+      <c r="I21" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J21" s="23" t="s">
@@ -6107,10 +6107,10 @@
       <c r="G22" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H22" s="28" t="s">
+      <c r="H22" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="I22" s="29" t="s">
+      <c r="I22" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J22" s="23" t="s">
@@ -6137,10 +6137,10 @@
       <c r="G23" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H23" s="28" t="s">
+      <c r="H23" s="27" t="s">
         <v>247</v>
       </c>
-      <c r="I23" s="29" t="s">
+      <c r="I23" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J23" s="23"/>
@@ -6165,10 +6165,10 @@
       <c r="G24" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H24" s="28" t="s">
+      <c r="H24" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="I24" s="29" t="s">
+      <c r="I24" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J24" s="23"/>
@@ -6193,10 +6193,10 @@
       <c r="G25" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H25" s="28" t="s">
+      <c r="H25" s="27" t="s">
         <v>265</v>
       </c>
-      <c r="I25" s="29" t="s">
+      <c r="I25" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J25" s="23"/>
@@ -6222,7 +6222,7 @@
         <v>354</v>
       </c>
       <c r="H26" s="23"/>
-      <c r="I26" s="29" t="s">
+      <c r="I26" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J26" s="23" t="s">
@@ -6249,10 +6249,10 @@
       <c r="G27" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H27" s="28" t="s">
+      <c r="H27" s="27" t="s">
         <v>280</v>
       </c>
-      <c r="I27" s="29" t="s">
+      <c r="I27" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J27" s="23"/>
@@ -6277,10 +6277,10 @@
       <c r="G28" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H28" s="28" t="s">
+      <c r="H28" s="27" t="s">
         <v>287</v>
       </c>
-      <c r="I28" s="29" t="s">
+      <c r="I28" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J28" s="23" t="s">
@@ -6307,10 +6307,10 @@
       <c r="G29" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H29" s="28" t="s">
+      <c r="H29" s="27" t="s">
         <v>289</v>
       </c>
-      <c r="I29" s="29" t="s">
+      <c r="I29" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J29" s="23"/>
@@ -6335,10 +6335,10 @@
       <c r="G30" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H30" s="28" t="s">
+      <c r="H30" s="27" t="s">
         <v>292</v>
       </c>
-      <c r="I30" s="29" t="s">
+      <c r="I30" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J30" s="23"/>
@@ -6363,10 +6363,10 @@
       <c r="G31" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H31" s="28" t="s">
+      <c r="H31" s="27" t="s">
         <v>300</v>
       </c>
-      <c r="I31" s="29" t="s">
+      <c r="I31" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J31" s="23" t="s">
@@ -6393,10 +6393,10 @@
       <c r="G32" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H32" s="28" t="s">
+      <c r="H32" s="27" t="s">
         <v>298</v>
       </c>
-      <c r="I32" s="29" t="s">
+      <c r="I32" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J32" s="23" t="s">
@@ -6425,10 +6425,10 @@
       <c r="G33" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H33" s="28" t="s">
+      <c r="H33" s="27" t="s">
         <v>314</v>
       </c>
-      <c r="I33" s="29" t="s">
+      <c r="I33" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J33" s="23" t="s">
@@ -6455,10 +6455,10 @@
       <c r="G34" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H34" s="28" t="s">
+      <c r="H34" s="27" t="s">
         <v>303</v>
       </c>
-      <c r="I34" s="29" t="s">
+      <c r="I34" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J34" s="23" t="s">
@@ -6487,10 +6487,10 @@
       <c r="G35" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H35" s="28" t="s">
+      <c r="H35" s="27" t="s">
         <v>309</v>
       </c>
-      <c r="I35" s="29" t="s">
+      <c r="I35" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J35" s="23" t="s">
@@ -6517,10 +6517,10 @@
       <c r="G36" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H36" s="28" t="s">
+      <c r="H36" s="27" t="s">
         <v>311</v>
       </c>
-      <c r="I36" s="29" t="s">
+      <c r="I36" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J36" s="23"/>
@@ -6545,10 +6545,10 @@
       <c r="G37" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="H37" s="28" t="s">
+      <c r="H37" s="27" t="s">
         <v>460</v>
       </c>
-      <c r="I37" s="29" t="s">
+      <c r="I37" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J37" s="23" t="s">
@@ -6575,10 +6575,10 @@
       <c r="G38" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H38" s="28" t="s">
+      <c r="H38" s="27" t="s">
         <v>323</v>
       </c>
-      <c r="I38" s="29" t="s">
+      <c r="I38" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J38" s="23"/>
@@ -6603,10 +6603,10 @@
       <c r="G39" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="H39" s="28" t="s">
+      <c r="H39" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="I39" s="29" t="s">
+      <c r="I39" s="28" t="s">
         <v>84</v>
       </c>
       <c r="J39" s="23"/>
@@ -6625,7 +6625,7 @@
       <formula>"In progress"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" sqref="I2:I39" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Not started,In progress,Done,Skipped"</formula1>
       <formula2>0</formula2>
@@ -6842,15 +6842,15 @@
       <c r="D2" s="23" t="s">
         <v>497</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="38"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="23" t="str">
         <f t="shared" ref="G2:G13" ca="1" si="0">IF(F2="","",IF(TODAY()-F2&lt;=365,"Yes","No: check another course"))</f>
         <v/>
       </c>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29" t="s">
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K2" s="23" t="s">
@@ -6870,15 +6870,15 @@
       <c r="D3" s="23" t="s">
         <v>500</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="38"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="37"/>
       <c r="G3" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29" t="s">
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K3" s="23" t="s">
@@ -6898,15 +6898,15 @@
       <c r="D4" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="E4" s="29"/>
-      <c r="F4" s="38"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="37"/>
       <c r="G4" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29" t="s">
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K4" s="23" t="s">
@@ -6926,15 +6926,15 @@
       <c r="D5" s="23" t="s">
         <v>507</v>
       </c>
-      <c r="E5" s="29"/>
-      <c r="F5" s="38"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="37"/>
       <c r="G5" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29" t="s">
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K5" s="23" t="s">
@@ -6954,15 +6954,15 @@
       <c r="D6" s="23" t="s">
         <v>509</v>
       </c>
-      <c r="E6" s="29"/>
-      <c r="F6" s="38"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="37"/>
       <c r="G6" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29" t="s">
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K6" s="23" t="s">
@@ -6982,15 +6982,15 @@
       <c r="D7" s="23" t="s">
         <v>512</v>
       </c>
-      <c r="E7" s="29"/>
-      <c r="F7" s="38"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="37"/>
       <c r="G7" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29" t="s">
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K7" s="23" t="s">
@@ -7010,15 +7010,15 @@
       <c r="D8" s="23" t="s">
         <v>514</v>
       </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="38"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="37"/>
       <c r="G8" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29" t="s">
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K8" s="23" t="s">
@@ -7038,15 +7038,15 @@
       <c r="D9" s="23" t="s">
         <v>517</v>
       </c>
-      <c r="E9" s="29"/>
-      <c r="F9" s="38"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="37"/>
       <c r="G9" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29" t="s">
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K9" s="23" t="s">
@@ -7066,15 +7066,15 @@
       <c r="D10" s="23" t="s">
         <v>519</v>
       </c>
-      <c r="E10" s="29"/>
-      <c r="F10" s="38"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="37"/>
       <c r="G10" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29" t="s">
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K10" s="23" t="s">
@@ -7094,15 +7094,15 @@
       <c r="D11" s="23" t="s">
         <v>522</v>
       </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="38"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="37"/>
       <c r="G11" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29" t="s">
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K11" s="23" t="s">
@@ -7122,15 +7122,15 @@
       <c r="D12" s="23" t="s">
         <v>524</v>
       </c>
-      <c r="E12" s="29"/>
-      <c r="F12" s="38"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="37"/>
       <c r="G12" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H12" s="29"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="29" t="s">
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K12" s="23" t="s">
@@ -7150,15 +7150,15 @@
       <c r="D13" s="23" t="s">
         <v>528</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="38"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="37"/>
       <c r="G13" s="23" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29" t="s">
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28" t="s">
         <v>84</v>
       </c>
       <c r="K13" s="23" t="s">
@@ -7226,22 +7226,22 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="28" t="s">
         <v>538</v>
       </c>
-      <c r="B2" s="29">
+      <c r="B2" s="28">
         <v>1</v>
       </c>
-      <c r="C2" s="38">
+      <c r="C2" s="37">
         <v>46374</v>
       </c>
-      <c r="D2" s="39">
+      <c r="D2" s="38">
         <v>0.68</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="28" t="s">
         <v>539</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="28" t="s">
         <v>540</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -7249,319 +7249,319 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
       <c r="H3" s="2" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="29"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="29"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="29"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
+      <c r="A28" s="28"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
+      <c r="A29" s="28"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="29"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="29"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="29"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="29"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
+      <c r="A35" s="28"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="29"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="29"/>
+      <c r="A36" s="28"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="29"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="38"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
+      <c r="A37" s="28"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="29"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="39"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
+      <c r="A38" s="28"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="29"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="29"/>
+      <c r="A39" s="28"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="29"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="29"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
+      <c r="A41" s="28"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -7622,7 +7622,7 @@
       <c r="B2" s="23">
         <v>1</v>
       </c>
-      <c r="C2" s="31">
+      <c r="C2" s="30">
         <f>Dashboard!$B$4+B2*7-3</f>
         <v>46318</v>
       </c>
@@ -7635,10 +7635,10 @@
       <c r="F2" s="23" t="s">
         <v>551</v>
       </c>
-      <c r="G2" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2" s="29"/>
+      <c r="G2" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
@@ -7647,7 +7647,7 @@
       <c r="B3" s="23">
         <v>1</v>
       </c>
-      <c r="C3" s="31">
+      <c r="C3" s="30">
         <f>Dashboard!$B$4+B3*7-3</f>
         <v>46318</v>
       </c>
@@ -7660,10 +7660,10 @@
       <c r="F3" s="23" t="s">
         <v>555</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H3" s="29"/>
+      <c r="G3" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -7672,7 +7672,7 @@
       <c r="B4" s="23">
         <v>2</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="30">
         <f>Dashboard!$B$4+B4*7-3</f>
         <v>46325</v>
       </c>
@@ -7685,10 +7685,10 @@
       <c r="F4" s="23" t="s">
         <v>559</v>
       </c>
-      <c r="G4" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H4" s="29"/>
+      <c r="G4" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
@@ -7697,7 +7697,7 @@
       <c r="B5" s="23">
         <v>2</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="30">
         <f>Dashboard!$B$4+B5*7-3</f>
         <v>46325</v>
       </c>
@@ -7710,10 +7710,10 @@
       <c r="F5" s="23" t="s">
         <v>562</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H5" s="29"/>
+      <c r="G5" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
@@ -7722,7 +7722,7 @@
       <c r="B6" s="23">
         <v>3</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="30">
         <f>Dashboard!$B$4+B6*7-3</f>
         <v>46332</v>
       </c>
@@ -7735,10 +7735,10 @@
       <c r="F6" s="23" t="s">
         <v>566</v>
       </c>
-      <c r="G6" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H6" s="29"/>
+      <c r="G6" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
@@ -7747,7 +7747,7 @@
       <c r="B7" s="23">
         <v>3</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="30">
         <f>Dashboard!$B$4+B7*7-3</f>
         <v>46332</v>
       </c>
@@ -7760,10 +7760,10 @@
       <c r="F7" s="23" t="s">
         <v>570</v>
       </c>
-      <c r="G7" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H7" s="29"/>
+      <c r="G7" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H7" s="28"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
@@ -7772,7 +7772,7 @@
       <c r="B8" s="23">
         <v>4</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="30">
         <f>Dashboard!$B$4+B8*7-3</f>
         <v>46339</v>
       </c>
@@ -7785,10 +7785,10 @@
       <c r="F8" s="23" t="s">
         <v>573</v>
       </c>
-      <c r="G8" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H8" s="29"/>
+      <c r="G8" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H8" s="28"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
@@ -7797,7 +7797,7 @@
       <c r="B9" s="23">
         <v>4</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="30">
         <f>Dashboard!$B$4+B9*7-3</f>
         <v>46339</v>
       </c>
@@ -7810,10 +7810,10 @@
       <c r="F9" s="23" t="s">
         <v>576</v>
       </c>
-      <c r="G9" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H9" s="29"/>
+      <c r="G9" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
@@ -7822,7 +7822,7 @@
       <c r="B10" s="23">
         <v>5</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="30">
         <f>Dashboard!$B$4+B10*7-3</f>
         <v>46346</v>
       </c>
@@ -7835,10 +7835,10 @@
       <c r="F10" s="23" t="s">
         <v>578</v>
       </c>
-      <c r="G10" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H10" s="29"/>
+      <c r="G10" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H10" s="28"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="23" t="s">
@@ -7847,7 +7847,7 @@
       <c r="B11" s="23">
         <v>6</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="30">
         <f>Dashboard!$B$4+B11*7-3</f>
         <v>46353</v>
       </c>
@@ -7860,10 +7860,10 @@
       <c r="F11" s="23" t="s">
         <v>580</v>
       </c>
-      <c r="G11" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="29"/>
+      <c r="G11" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H11" s="28"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
@@ -7872,7 +7872,7 @@
       <c r="B12" s="23">
         <v>7</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="30">
         <f>Dashboard!$B$4+B12*7-3</f>
         <v>46360</v>
       </c>
@@ -7885,10 +7885,10 @@
       <c r="F12" s="23" t="s">
         <v>582</v>
       </c>
-      <c r="G12" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H12" s="29"/>
+      <c r="G12" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="23" t="s">
@@ -7897,7 +7897,7 @@
       <c r="B13" s="23">
         <v>10</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="30">
         <f>Dashboard!$B$4+B13*7-3</f>
         <v>46381</v>
       </c>
@@ -7910,10 +7910,10 @@
       <c r="F13" s="23" t="s">
         <v>584</v>
       </c>
-      <c r="G13" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H13" s="29"/>
+      <c r="G13" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
@@ -7922,7 +7922,7 @@
       <c r="B14" s="23">
         <v>11</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="30">
         <f>Dashboard!$B$4+B14*7-3</f>
         <v>46388</v>
       </c>
@@ -7935,10 +7935,10 @@
       <c r="F14" s="23" t="s">
         <v>586</v>
       </c>
-      <c r="G14" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H14" s="29"/>
+      <c r="G14" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" s="28"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
@@ -7947,7 +7947,7 @@
       <c r="B15" s="23">
         <v>12</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="30">
         <f>Dashboard!$B$4+B15*7-3</f>
         <v>46395</v>
       </c>
@@ -7960,10 +7960,10 @@
       <c r="F15" s="23" t="s">
         <v>588</v>
       </c>
-      <c r="G15" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="29"/>
+      <c r="G15" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
@@ -7972,7 +7972,7 @@
       <c r="B16" s="23">
         <v>13</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="30">
         <f>Dashboard!$B$4+B16*7-3</f>
         <v>46402</v>
       </c>
@@ -7985,10 +7985,10 @@
       <c r="F16" s="23" t="s">
         <v>590</v>
       </c>
-      <c r="G16" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H16" s="29"/>
+      <c r="G16" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="23" t="s">
@@ -7997,7 +7997,7 @@
       <c r="B17" s="23">
         <v>14</v>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="30">
         <f>Dashboard!$B$4+B17*7-3</f>
         <v>46409</v>
       </c>
@@ -8010,10 +8010,10 @@
       <c r="F17" s="23" t="s">
         <v>592</v>
       </c>
-      <c r="G17" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="29"/>
+      <c r="G17" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
@@ -8022,7 +8022,7 @@
       <c r="B18" s="23">
         <v>15</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="30">
         <f>Dashboard!$B$4+B18*7-3</f>
         <v>46416</v>
       </c>
@@ -8035,10 +8035,10 @@
       <c r="F18" s="23" t="s">
         <v>594</v>
       </c>
-      <c r="G18" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H18" s="29"/>
+      <c r="G18" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="28"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="23" t="s">
@@ -8047,7 +8047,7 @@
       <c r="B19" s="23">
         <v>16</v>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="30">
         <f>Dashboard!$B$4+B19*7-3</f>
         <v>46423</v>
       </c>
@@ -8060,10 +8060,10 @@
       <c r="F19" s="23" t="s">
         <v>596</v>
       </c>
-      <c r="G19" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H19" s="29"/>
+      <c r="G19" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H19" s="28"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="23" t="s">
@@ -8072,7 +8072,7 @@
       <c r="B20" s="23">
         <v>17</v>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="30">
         <f>Dashboard!$B$4+B20*7-3</f>
         <v>46430</v>
       </c>
@@ -8085,10 +8085,10 @@
       <c r="F20" s="23" t="s">
         <v>598</v>
       </c>
-      <c r="G20" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H20" s="29"/>
+      <c r="G20" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="23" t="s">
@@ -8097,7 +8097,7 @@
       <c r="B21" s="23">
         <v>18</v>
       </c>
-      <c r="C21" s="31">
+      <c r="C21" s="30">
         <f>Dashboard!$B$4+B21*7-3</f>
         <v>46437</v>
       </c>
@@ -8110,10 +8110,10 @@
       <c r="F21" s="23" t="s">
         <v>600</v>
       </c>
-      <c r="G21" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H21" s="29"/>
+      <c r="G21" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="23" t="s">
@@ -8122,7 +8122,7 @@
       <c r="B22" s="23">
         <v>19</v>
       </c>
-      <c r="C22" s="31">
+      <c r="C22" s="30">
         <f>Dashboard!$B$4+B22*7-3</f>
         <v>46444</v>
       </c>
@@ -8135,10 +8135,10 @@
       <c r="F22" s="23" t="s">
         <v>295</v>
       </c>
-      <c r="G22" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H22" s="29"/>
+      <c r="G22" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
@@ -8147,7 +8147,7 @@
       <c r="B23" s="23">
         <v>20</v>
       </c>
-      <c r="C23" s="31">
+      <c r="C23" s="30">
         <f>Dashboard!$B$4+B23*7-3</f>
         <v>46451</v>
       </c>
@@ -8160,10 +8160,10 @@
       <c r="F23" s="23" t="s">
         <v>603</v>
       </c>
-      <c r="G23" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H23" s="29"/>
+      <c r="G23" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="23" t="s">
@@ -8172,7 +8172,7 @@
       <c r="B24" s="23">
         <v>21</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="30">
         <f>Dashboard!$B$4+B24*7-3</f>
         <v>46458</v>
       </c>
@@ -8185,10 +8185,10 @@
       <c r="F24" s="23" t="s">
         <v>605</v>
       </c>
-      <c r="G24" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H24" s="29"/>
+      <c r="G24" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H24" s="28"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
@@ -8197,7 +8197,7 @@
       <c r="B25" s="23">
         <v>22</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="30">
         <f>Dashboard!$B$4+B25*7-3</f>
         <v>46465</v>
       </c>
@@ -8210,10 +8210,10 @@
       <c r="F25" s="23" t="s">
         <v>608</v>
       </c>
-      <c r="G25" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H25" s="29"/>
+      <c r="G25" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="23" t="s">
@@ -8222,7 +8222,7 @@
       <c r="B26" s="23">
         <v>22</v>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="30">
         <f>Dashboard!$B$4+B26*7-3</f>
         <v>46465</v>
       </c>
@@ -8235,10 +8235,10 @@
       <c r="F26" s="23" t="s">
         <v>611</v>
       </c>
-      <c r="G26" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H26" s="29"/>
+      <c r="G26" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H26" s="28"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="23" t="s">
@@ -8247,7 +8247,7 @@
       <c r="B27" s="23">
         <v>22</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="30">
         <f>Dashboard!$B$4+B27*7-3</f>
         <v>46465</v>
       </c>
@@ -8260,10 +8260,10 @@
       <c r="F27" s="23" t="s">
         <v>615</v>
       </c>
-      <c r="G27" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H27" s="29"/>
+      <c r="G27" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" s="28"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="23" t="s">
@@ -8272,7 +8272,7 @@
       <c r="B28" s="23">
         <v>23</v>
       </c>
-      <c r="C28" s="31">
+      <c r="C28" s="30">
         <f>Dashboard!$B$4+B28*7-3</f>
         <v>46472</v>
       </c>
@@ -8285,10 +8285,10 @@
       <c r="F28" s="23" t="s">
         <v>618</v>
       </c>
-      <c r="G28" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H28" s="29"/>
+      <c r="G28" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="28"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
@@ -8297,7 +8297,7 @@
       <c r="B29" s="23">
         <v>23</v>
       </c>
-      <c r="C29" s="31">
+      <c r="C29" s="30">
         <f>Dashboard!$B$4+B29*7-3</f>
         <v>46472</v>
       </c>
@@ -8310,10 +8310,10 @@
       <c r="F29" s="23" t="s">
         <v>622</v>
       </c>
-      <c r="G29" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H29" s="29"/>
+      <c r="G29" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" s="28"/>
     </row>
     <row r="30" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
@@ -8322,7 +8322,7 @@
       <c r="B30" s="23">
         <v>8</v>
       </c>
-      <c r="C30" s="31">
+      <c r="C30" s="30">
         <f>Dashboard!$B$4+B30*7-3</f>
         <v>46367</v>
       </c>
@@ -8335,10 +8335,10 @@
       <c r="F30" s="23" t="s">
         <v>624</v>
       </c>
-      <c r="G30" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H30" s="29"/>
+      <c r="G30" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
@@ -8347,7 +8347,7 @@
       <c r="B31" s="23">
         <v>9</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="30">
         <f>Dashboard!$B$4+B31*7-3</f>
         <v>46374</v>
       </c>
@@ -8360,10 +8360,10 @@
       <c r="F31" s="23" t="s">
         <v>626</v>
       </c>
-      <c r="G31" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="H31" s="29"/>
+      <c r="G31" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="H31" s="28"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G29">

</xml_diff>